<commit_message>
Generate ARR demo baseline from workbook ingestion
</commit_message>
<xml_diff>
--- a/apps/arr-v2/frontend/public/demo/arr-v2-demo-import.xlsx
+++ b/apps/arr-v2/frontend/public/demo/arr-v2-demo-import.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>Customer</t>
   </si>
@@ -343,6 +343,57 @@
   </si>
   <si>
     <t>2027-03-19</t>
+  </si>
+  <si>
+    <t>Cascade BioLabs</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>INV-1320</t>
+  </si>
+  <si>
+    <t>Life Sciences Analytics Cloud</t>
+  </si>
+  <si>
+    <t>New life-sciences platform subscription</t>
+  </si>
+  <si>
+    <t>2027-03-31</t>
+  </si>
+  <si>
+    <t>Life Sciences</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>INV-1327</t>
+  </si>
+  <si>
+    <t>Route Optimization Add-On</t>
+  </si>
+  <si>
+    <t>New route optimization expansion</t>
+  </si>
+  <si>
+    <t>2027-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>INV-1331</t>
+  </si>
+  <si>
+    <t>Care Quality Benchmarking</t>
+  </si>
+  <si>
+    <t>New care-quality benchmarking expansion</t>
+  </si>
+  <si>
+    <t>2027-04-19</t>
   </si>
   <si>
     <t>Dashboard Subscription</t>
@@ -1110,6 +1161,138 @@
         <v>31</v>
       </c>
       <c r="N17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" t="s">
+        <v>114</v>
+      </c>
+      <c r="F18" t="s">
+        <v>115</v>
+      </c>
+      <c r="G18">
+        <v>12</v>
+      </c>
+      <c r="H18">
+        <v>24500</v>
+      </c>
+      <c r="I18">
+        <v>294000</v>
+      </c>
+      <c r="J18" t="s">
+        <v>112</v>
+      </c>
+      <c r="K18" t="s">
+        <v>116</v>
+      </c>
+      <c r="L18" t="s">
+        <v>21</v>
+      </c>
+      <c r="M18" t="s">
+        <v>117</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" t="s">
+        <v>120</v>
+      </c>
+      <c r="F19" t="s">
+        <v>121</v>
+      </c>
+      <c r="G19">
+        <v>12</v>
+      </c>
+      <c r="H19">
+        <v>8500</v>
+      </c>
+      <c r="I19">
+        <v>102000</v>
+      </c>
+      <c r="J19" t="s">
+        <v>118</v>
+      </c>
+      <c r="K19" t="s">
+        <v>122</v>
+      </c>
+      <c r="L19" t="s">
+        <v>21</v>
+      </c>
+      <c r="M19" t="s">
+        <v>42</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" t="s">
+        <v>126</v>
+      </c>
+      <c r="G20">
+        <v>12</v>
+      </c>
+      <c r="H20">
+        <v>9200</v>
+      </c>
+      <c r="I20">
+        <v>110400</v>
+      </c>
+      <c r="J20" t="s">
+        <v>123</v>
+      </c>
+      <c r="K20" t="s">
+        <v>127</v>
+      </c>
+      <c r="L20" t="s">
+        <v>21</v>
+      </c>
+      <c r="M20" t="s">
+        <v>22</v>
+      </c>
+      <c r="N20">
         <v>0</v>
       </c>
     </row>
@@ -1125,13 +1308,13 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="C1" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="D1" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="E1" t="s">
         <v>105</v>
@@ -1142,7 +1325,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -1150,7 +1333,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4">
@@ -1158,7 +1341,7 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
@@ -1166,7 +1349,7 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6">
@@ -1174,7 +1357,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7">
@@ -1182,7 +1365,7 @@
         <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8">
@@ -1190,7 +1373,7 @@
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
@@ -1198,7 +1381,7 @@
         <v>58</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
@@ -1206,7 +1389,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11">
@@ -1214,7 +1397,7 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12">
@@ -1222,7 +1405,7 @@
         <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13">
@@ -1230,7 +1413,7 @@
         <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14">
@@ -1238,7 +1421,7 @@
         <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15">
@@ -1246,7 +1429,7 @@
         <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16">
@@ -1254,7 +1437,7 @@
         <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17">
@@ -1262,7 +1445,31 @@
         <v>108</v>
       </c>
       <c r="B17" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
         <v>114</v>
+      </c>
+      <c r="B18" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1274,39 +1481,39 @@
   <sheetData>
     <row r="1">
       <c r="B1" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="C4" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6">
@@ -1314,7 +1521,7 @@
         <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>